<commit_message>
feat(divergent-universe): add runtime foundation and partial gameplay
Include the coupled Sora 0.6.1 reference and decision catalogs, runtime rules, replay adapters, tests and current-state documentation.

This is an incomplete runtime, not a release acceptance claim. The current ledger retains 6578 pending obligations; repository-audit ledger drift and production domain-deck binding remain unresolved.

Record the authorized per-batch commit workflow and ignore local Python bytecode.
</commit_message>
<xml_diff>
--- a/config/divergent-universe-generated/templates/DivergentUniverse.xlsx
+++ b/config/divergent-universe-generated/templates/DivergentUniverse.xlsx
@@ -91,16 +91,16 @@
     <t>id</t>
   </si>
   <si>
-    <t>@scope</t>
-  </si>
-  <si>
-    <t>all</t>
+    <t>@groups</t>
+  </si>
+  <si>
+    <t>common</t>
   </si>
   <si>
     <t>@schema</t>
   </si>
   <si>
-    <t>87e82545945935af</t>
+    <t>b4964060ee2752ad</t>
   </si>
   <si>
     <t>#name</t>
@@ -199,7 +199,7 @@
     <t>optional&lt;list&lt;ref&lt;DivergentUniverseFinishConditions.id&gt;&gt;&gt;</t>
   </si>
   <si>
-    <t>#scope</t>
+    <t>#groups</t>
   </si>
   <si>
     <t>#input</t>
@@ -235,7 +235,7 @@
     <t>DivergentUniverseModules</t>
   </si>
   <si>
-    <t>5a18d35a75bf680e</t>
+    <t>b99d201e047380dc</t>
   </si>
   <si>
     <t>sub_mode</t>
@@ -253,7 +253,7 @@
     <t>DivergentUniverseEntries</t>
   </si>
   <si>
-    <t>bc5fde22f56064bf</t>
+    <t>8c5fc0ebc8496993</t>
   </si>
   <si>
     <t>entry_kind</t>
@@ -265,7 +265,7 @@
     <t>DivergentUniverseFinishConditions</t>
   </si>
   <si>
-    <t>784f78fb4e12fb05</t>
+    <t>73e50a31ff00f359</t>
   </si>
   <si>
     <t>condition_kind</t>
@@ -280,7 +280,7 @@
     <t>DivergentUniverseAreas</t>
   </si>
   <si>
-    <t>38f7ba402c6f1946</t>
+    <t>b357b25055324a7a</t>
   </si>
   <si>
     <t>difficulty_ids</t>
@@ -304,7 +304,7 @@
     <t>DivergentUniverseDifficulties</t>
   </si>
   <si>
-    <t>9190266d8ad95c33</t>
+    <t>4cc974217ed98823</t>
   </si>
   <si>
     <t>level_list</t>
@@ -319,7 +319,7 @@
     <t>DivergentUniverseLayers</t>
   </si>
   <si>
-    <t>d7bd0e8c8d275115</t>
+    <t>fcee08e2d37619e5</t>
   </si>
   <si>
     <t>layer_number</t>
@@ -331,7 +331,7 @@
     <t>DivergentUniverseLayerRooms</t>
   </si>
   <si>
-    <t>055c66c8f465f76d</t>
+    <t>ed3969cb8ae20821</t>
   </si>
   <si>
     <t>layer_id</t>
@@ -349,7 +349,7 @@
     <t>DivergentUniverseRooms</t>
   </si>
   <si>
-    <t>5aac27c2d16d723c</t>
+    <t>9e29c5b490793224</t>
   </si>
   <si>
     <t>room_type</t>
@@ -364,7 +364,7 @@
     <t>DivergentUniverseStageFlow</t>
   </si>
   <si>
-    <t>b421d44bb4eb829d</t>
+    <t>c1a1264299e64549</t>
   </si>
   <si>
     <t>entry_id</t>
@@ -382,7 +382,7 @@
     <t>DivergentUniverseCyclicalChallenges</t>
   </si>
   <si>
-    <t>7c426538bf1cd2c9</t>
+    <t>8066d74bb09f7435</t>
   </si>
   <si>
     <t>area_id</t>
@@ -403,7 +403,7 @@
     <t>DivergentUniverseProtocols</t>
   </si>
   <si>
-    <t>593a1e5ac5317de5</t>
+    <t>c9d47b8a010f50d3</t>
   </si>
   <si>
     <t>protocol_level</t>
@@ -421,7 +421,7 @@
     <t>DivergentUniverseAstronomicalDivisions</t>
   </si>
   <si>
-    <t>e96c2579e6252c42</t>
+    <t>8b2c343e5039de58</t>
   </si>
   <si>
     <t>division_level</t>
@@ -436,7 +436,7 @@
     <t>DivergentUniverseStarPioneerPractice</t>
   </si>
   <si>
-    <t>11c47b469312c131</t>
+    <t>64120559ea1742ed</t>
   </si>
   <si>
     <t>mode_kind</t>
@@ -448,7 +448,7 @@
     <t>DivergentUniverseCognoculi</t>
   </si>
   <si>
-    <t>6942c546e656c57e</t>
+    <t>4c36418d97669e8a</t>
   </si>
   <si>
     <t>source_locator</t>
@@ -463,7 +463,7 @@
     <t>DivergentUniverseArithmeticMappingEligibility</t>
   </si>
   <si>
-    <t>20b8a6b6ab3d347b</t>
+    <t>31dbeefdb94fe731</t>
   </si>
   <si>
     <t>avatar_id</t>
@@ -478,7 +478,7 @@
     <t>DivergentUniverseArithmeticMappingBuilds</t>
   </si>
   <si>
-    <t>ecc3c87378bd6a43</t>
+    <t>ae4e21879ac4aa19</t>
   </si>
   <si>
     <t>level</t>
@@ -499,7 +499,7 @@
     <t>DivergentUniverseArithmeticMappingRules</t>
   </si>
   <si>
-    <t>beb0cd1360417f68</t>
+    <t>04995c69a9d1c8b0</t>
   </si>
   <si>
     <t>selection_timing</t>
@@ -517,7 +517,7 @@
     <t>DivergentUniverseEquations</t>
   </si>
   <si>
-    <t>6f37548f1bce71d9</t>
+    <t>c1a3b23260d6cdc3</t>
   </si>
   <si>
     <t>recipe_id</t>
@@ -541,7 +541,7 @@
     <t>DivergentUniverseEquationRecipes</t>
   </si>
   <si>
-    <t>ffccd420ad25256b</t>
+    <t>e349b336b19c5c63</t>
   </si>
   <si>
     <t>equation_id</t>
@@ -562,7 +562,7 @@
     <t>DivergentUniverseEquationCategories</t>
   </si>
   <si>
-    <t>40bba903f15e4798</t>
+    <t>01a30efd0bcdef16</t>
   </si>
   <si>
     <t>offer_rules</t>
@@ -574,7 +574,7 @@
     <t>DivergentUniverseEquationOffers</t>
   </si>
   <si>
-    <t>2b7a5639135c3eab</t>
+    <t>bf48c09c8b4af56f</t>
   </si>
   <si>
     <t>candidate_ids</t>
@@ -592,7 +592,7 @@
     <t>DivergentUniverseEquationProgress</t>
   </si>
   <si>
-    <t>d782c6c83713c22e</t>
+    <t>1892bece50603eb8</t>
   </si>
   <si>
     <t>contribution_rule</t>
@@ -604,7 +604,7 @@
     <t>DivergentUniverseEquationExpansionStates</t>
   </si>
   <si>
-    <t>b67a095200ff9f5b</t>
+    <t>ba539e99897e2c73</t>
   </si>
   <si>
     <t>state</t>
@@ -619,7 +619,7 @@
     <t>DivergentUniverseEquationEffects</t>
   </si>
   <si>
-    <t>95a9a61be6942680</t>
+    <t>bd15aa1138fd42ae</t>
   </si>
   <si>
     <t>keyword_ids</t>
@@ -631,7 +631,7 @@
     <t>DivergentUniverseEquationReplacementRules</t>
   </si>
   <si>
-    <t>87b69c662e60a876</t>
+    <t>6d323aa272ce3382</t>
   </si>
   <si>
     <t>operation</t>
@@ -646,7 +646,7 @@
     <t>DivergentUniverseBlessingPaths</t>
   </si>
   <si>
-    <t>e722d7554fac0fe4</t>
+    <t>8ce59944dc93a3fc</t>
   </si>
   <si>
     <t>path_id</t>
@@ -661,7 +661,7 @@
     <t>DivergentUniverseBlessings</t>
   </si>
   <si>
-    <t>3f7f44268d16154a</t>
+    <t>cc27f69f33a19150</t>
   </si>
   <si>
     <t>level_ids</t>
@@ -670,7 +670,7 @@
     <t>DivergentUniverseBlessingLevels</t>
   </si>
   <si>
-    <t>20ea69f4e8d43107</t>
+    <t>9ad437669888abdb</t>
   </si>
   <si>
     <t>blessing_id</t>
@@ -682,7 +682,7 @@
     <t>DivergentUniverseBlessingGroups</t>
   </si>
   <si>
-    <t>08c18ff88964ceff</t>
+    <t>75ab69d1321d6409</t>
   </si>
   <si>
     <t>selection_policy</t>
@@ -691,7 +691,7 @@
     <t>DivergentUniverseBlessingRewriteRules</t>
   </si>
   <si>
-    <t>83836f6870d09830</t>
+    <t>f2d4b89d933e6d22</t>
   </si>
   <si>
     <t>input_blessing_id</t>
@@ -712,7 +712,7 @@
     <t>DivergentUniverseBlessingEquationContributions</t>
   </si>
   <si>
-    <t>37ff39692102e015</t>
+    <t>0452a8ca89668c53</t>
   </si>
   <si>
     <t>equation_ids</t>
@@ -727,7 +727,7 @@
     <t>DivergentUniverseCurios</t>
   </si>
   <si>
-    <t>75c158400c465264</t>
+    <t>8127aa6d653f6bf0</t>
   </si>
   <si>
     <t>state_ids</t>
@@ -739,7 +739,7 @@
     <t>DivergentUniverseCurioStates</t>
   </si>
   <si>
-    <t>53004453d83392ff</t>
+    <t>2dbdac7323631c31</t>
   </si>
   <si>
     <t>curio_id</t>
@@ -754,7 +754,7 @@
     <t>DivergentUniverseCurioGroups</t>
   </si>
   <si>
-    <t>91b996eba7358d2c</t>
+    <t>0dc9f741dd8aba98</t>
   </si>
   <si>
     <t>candidate_state_ids</t>
@@ -766,7 +766,7 @@
     <t>DivergentUniverseCurioLifecycleRules</t>
   </si>
   <si>
-    <t>f364887b6eff481b</t>
+    <t>52bf881e4f47df5b</t>
   </si>
   <si>
     <t>activation</t>
@@ -784,7 +784,7 @@
     <t>DivergentUniverseGrandMiracles</t>
   </si>
   <si>
-    <t>cc363dd44f5c3ba5</t>
+    <t>f8738c138824faeb</t>
   </si>
   <si>
     <t>display_id</t>
@@ -796,7 +796,7 @@
     <t>DivergentUniverseGrandMiracleEligibility</t>
   </si>
   <si>
-    <t>ec837451d97f2db6</t>
+    <t>447b51ba3cbfb12c</t>
   </si>
   <si>
     <t>grand_miracle_id</t>
@@ -814,7 +814,7 @@
     <t>DivergentUniverseGrandMiracleStates</t>
   </si>
   <si>
-    <t>18d8c21789a553f4</t>
+    <t>03155c56b20bcbce</t>
   </si>
   <si>
     <t>duration</t>
@@ -823,7 +823,7 @@
     <t>DivergentUniverseTitanTypes</t>
   </si>
   <si>
-    <t>10d8f2a9c89af50d</t>
+    <t>e50b51ef3e31d74b</t>
   </si>
   <si>
     <t>boon_ids</t>
@@ -835,7 +835,7 @@
     <t>DivergentUniverseTitanBoons</t>
   </si>
   <si>
-    <t>8ee36e31d71c0a37</t>
+    <t>34e1281d2a037843</t>
   </si>
   <si>
     <t>titan_type</t>
@@ -853,7 +853,7 @@
     <t>DivergentUniverseTitanTalents</t>
   </si>
   <si>
-    <t>4812097243aded9f</t>
+    <t>db1f197b7e02f903</t>
   </si>
   <si>
     <t>cost</t>
@@ -865,7 +865,7 @@
     <t>DivergentUniverseTitanChoices</t>
   </si>
   <si>
-    <t>a91949959fabe8e6</t>
+    <t>e83376058cc0e4be</t>
   </si>
   <si>
     <t>selection_count</t>
@@ -877,7 +877,7 @@
     <t>DivergentUniverseTitanContributions</t>
   </si>
   <si>
-    <t>35818620cb58cae9</t>
+    <t>d3336f9c9450da79</t>
   </si>
   <si>
     <t>scope</t>
@@ -889,7 +889,7 @@
     <t>DivergentUniverseWorkbenches</t>
   </si>
   <si>
-    <t>cfbc81d3a477a7c4</t>
+    <t>58149b2ada87ded2</t>
   </si>
   <si>
     <t>function_ids</t>
@@ -910,7 +910,7 @@
     <t>DivergentUniverseWorkbenchFunctions</t>
   </si>
   <si>
-    <t>d5467b80cc73442e</t>
+    <t>190a2ca736c343aa</t>
   </si>
   <si>
     <t>function_type</t>
@@ -928,7 +928,7 @@
     <t>DivergentUniverseGambleGroups</t>
   </si>
   <si>
-    <t>83d42c148e44eb8c</t>
+    <t>76b316d43f75d450</t>
   </si>
   <si>
     <t>group_type</t>
@@ -943,7 +943,7 @@
     <t>DivergentUniverseGambleUnits</t>
   </si>
   <si>
-    <t>5f8ceb1d686859a5</t>
+    <t>9c2979c16f43b725</t>
   </si>
   <si>
     <t>unit_type</t>
@@ -955,7 +955,7 @@
     <t>DivergentUniverseCurseChests</t>
   </si>
   <si>
-    <t>0dac35d4ad1d4df6</t>
+    <t>bcef8ace9dbac0fc</t>
   </si>
   <si>
     <t>chest_type</t>
@@ -967,7 +967,7 @@
     <t>DivergentUniverseCurrencies</t>
   </si>
   <si>
-    <t>452182101bdb41d6</t>
+    <t>6fa0ebd88ea4dc90</t>
   </si>
   <si>
     <t>gain_rules</t>
@@ -982,7 +982,7 @@
     <t>DivergentUniverseServiceRules</t>
   </si>
   <si>
-    <t>3c3543ffd2c70547</t>
+    <t>080139cc0d061135</t>
   </si>
   <si>
     <t>currency_id</t>
@@ -1003,7 +1003,7 @@
     <t>DivergentUniverseServiceOfferRules</t>
   </si>
   <si>
-    <t>a1ec343fcf33dfba</t>
+    <t>d64cb18bc62914fc</t>
   </si>
   <si>
     <t>service_id</t>
@@ -1015,7 +1015,7 @@
     <t>DivergentUniversePermanentTalents</t>
   </si>
   <si>
-    <t>7188e173c94e0e7b</t>
+    <t>b141bf3dd1078891</t>
   </si>
   <si>
     <t>prerequisite_ids</t>
@@ -1030,7 +1030,7 @@
     <t>DivergentUniverseUnlocks</t>
   </si>
   <si>
-    <t>fcea47d7ceda2571</t>
+    <t>9f680747a66af1ed</t>
   </si>
   <si>
     <t>finish_condition_id</t>
@@ -1045,7 +1045,7 @@
     <t>DivergentUniverseCommonConstants</t>
   </si>
   <si>
-    <t>83366f9c5d4d886f</t>
+    <t>501d52d0377d9c89</t>
   </si>
   <si>
     <t>value_kind</t>
@@ -1060,7 +1060,7 @@
     <t>DivergentUniverseWeeklyModifiers</t>
   </si>
   <si>
-    <t>8516ccfa5d76719a</t>
+    <t>a9fcf6f89fea8722</t>
   </si>
   <si>
     <t>content_ids</t>
@@ -1075,7 +1075,7 @@
     <t>DivergentUniverseRoomMarks</t>
   </si>
   <si>
-    <t>d29c4eb81adeadd4</t>
+    <t>70fb9b9a0ad4da94</t>
   </si>
   <si>
     <t>mark_kind</t>
@@ -1087,7 +1087,7 @@
     <t>DivergentUniverseProgressionEffects</t>
   </si>
   <si>
-    <t>db79ceddcfbf31b1</t>
+    <t>1ae670d758cde2fb</t>
   </si>
 </sst>
 </file>
@@ -1883,8 +1883,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -2274,8 +2274,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -2666,8 +2666,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -3057,8 +3057,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -3434,8 +3434,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -3825,8 +3825,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -4200,8 +4200,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -4576,8 +4576,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -4993,8 +4993,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -5384,8 +5384,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -5791,8 +5791,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -6180,8 +6180,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -6572,8 +6572,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -6948,8 +6948,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -7337,8 +7337,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -7729,8 +7729,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -8120,8 +8120,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -8510,8 +8510,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -8899,8 +8899,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -9274,8 +9274,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -9663,8 +9663,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -10054,8 +10054,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -10431,8 +10431,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -10806,8 +10806,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -11225,8 +11225,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -11632,8 +11632,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -12008,8 +12008,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -12399,8 +12399,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -12776,8 +12776,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -13195,8 +13195,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -13584,8 +13584,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -13975,8 +13975,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -14380,8 +14380,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -14756,8 +14756,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -15131,8 +15131,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -15536,8 +15536,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -15941,8 +15941,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -16348,8 +16348,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -16723,8 +16723,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -17104,8 +17104,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -17493,8 +17493,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -17868,8 +17868,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -18243,8 +18243,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -18618,8 +18618,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -19013,8 +19013,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -19402,8 +19402,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -19809,8 +19809,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -20212,8 +20212,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -20621,8 +20621,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -20999,8 +20999,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -21374,8 +21374,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -21763,8 +21763,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -22138,8 +22138,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -22500,8 +22500,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -22876,8 +22876,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -23238,8 +23238,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -23615,8 +23615,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>
@@ -23992,8 +23992,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
-      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: DivergentUniverse, Shared, OtherMode, Excluded, SharedCandidate" promptTitle="DuOwnership enum" prompt="Select a value from the dropdown." sqref="J8:J1007">
+      <formula1>"DivergentUniverse,Shared,OtherMode,Excluded,SharedCandidate"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Cataloged, Researched, DataReady, Blocked, Excluded" promptTitle="DuCoverageState enum" prompt="Select a value from the dropdown." sqref="K8:K1007">
       <formula1>"Cataloged,Researched,DataReady,Blocked,Excluded"</formula1>

</xml_diff>

<commit_message>
fix(divergent-universe): align weighted curio authoring and owned data
</commit_message>
<xml_diff>
--- a/config/divergent-universe-generated/templates/DivergentUniverse.xlsx
+++ b/config/divergent-universe-generated/templates/DivergentUniverse.xlsx
@@ -43,9 +43,9 @@
     <sheet name="T16_CurioStates" sheetId="34" r:id="rId34"/>
     <sheet name="T17_CurioGroups" sheetId="35" r:id="rId35"/>
     <sheet name="T18_CurioLifecycleRules" sheetId="36" r:id="rId36"/>
-    <sheet name="T19_GrandMiracles" sheetId="37" r:id="rId37"/>
-    <sheet name="T20_GrandMiracleEligibility" sheetId="38" r:id="rId38"/>
-    <sheet name="T21_GrandMiracleStates" sheetId="39" r:id="rId39"/>
+    <sheet name="T19_WeightedCurios" sheetId="37" r:id="rId37"/>
+    <sheet name="T20_WeightedCurioEligibility" sheetId="38" r:id="rId38"/>
+    <sheet name="T21_WeightedCurioStates" sheetId="39" r:id="rId39"/>
     <sheet name="T22_TitanTypes" sheetId="40" r:id="rId40"/>
     <sheet name="T23_TitanBoons" sheetId="41" r:id="rId41"/>
     <sheet name="T24_TitanTalents" sheetId="42" r:id="rId42"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5941" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5945" uniqueCount="341">
   <si>
     <t>@table</t>
   </si>
@@ -781,10 +781,13 @@
     <t>replacement</t>
   </si>
   <si>
-    <t>DivergentUniverseGrandMiracles</t>
-  </si>
-  <si>
-    <t>f8738c138824faeb</t>
+    <t>DivergentUniverseWeightedCurios</t>
+  </si>
+  <si>
+    <t>50b9f764d91309ef</t>
+  </si>
+  <si>
+    <t>content_kind</t>
   </si>
   <si>
     <t>display_id</t>
@@ -793,13 +796,16 @@
     <t>maze_buff_id</t>
   </si>
   <si>
-    <t>DivergentUniverseGrandMiracleEligibility</t>
-  </si>
-  <si>
-    <t>447b51ba3cbfb12c</t>
-  </si>
-  <si>
-    <t>grand_miracle_id</t>
+    <t>enum&lt;DuHexContentKind&gt;</t>
+  </si>
+  <si>
+    <t>DivergentUniverseWeightedCurioEligibility</t>
+  </si>
+  <si>
+    <t>5fe78dbd7895fc7c</t>
+  </si>
+  <si>
+    <t>weighted_curio_id</t>
   </si>
   <si>
     <t>character_path</t>
@@ -808,13 +814,13 @@
     <t>element</t>
   </si>
   <si>
-    <t>optional&lt;ref&lt;DivergentUniverseGrandMiracles.id&gt;&gt;</t>
-  </si>
-  <si>
-    <t>DivergentUniverseGrandMiracleStates</t>
-  </si>
-  <si>
-    <t>03155c56b20bcbce</t>
+    <t>optional&lt;ref&lt;DivergentUniverseWeightedCurios.id&gt;&gt;</t>
+  </si>
+  <si>
+    <t>DivergentUniverseWeightedCurioStates</t>
+  </si>
+  <si>
+    <t>610aec3cb1ae30d6</t>
   </si>
   <si>
     <t>duration</t>
@@ -13211,7 +13217,7 @@
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -13224,11 +13230,13 @@
     <col min="12" max="12" width="23.7109375" style="5" customWidth="1"/>
     <col min="13" max="13" width="32.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="22.7109375" style="5" customWidth="1"/>
-    <col min="15" max="19" width="16.7109375" style="5" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" style="5" customWidth="1"/>
+    <col min="16" max="16" width="22.7109375" style="5" customWidth="1"/>
+    <col min="17" max="20" width="16.7109375" style="5" customWidth="1"/>
+    <col min="21" max="21" width="12.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -13260,7 +13268,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="24" customHeight="1">
+    <row r="2" spans="1:21" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -13313,16 +13321,19 @@
         <v>239</v>
       </c>
       <c r="R2" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="S2" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="T2" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="T2" s="3" t="s">
+      <c r="U2" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:21">
       <c r="A3" s="4" t="s">
         <v>29</v>
       </c>
@@ -13375,16 +13386,19 @@
         <v>239</v>
       </c>
       <c r="R3" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="S3" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="T3" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="T3" s="5" t="s">
+      <c r="U3" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:21">
       <c r="A4" s="4" t="s">
         <v>30</v>
       </c>
@@ -13431,7 +13445,7 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>38</v>
+        <v>241</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>38</v>
@@ -13443,10 +13457,13 @@
         <v>38</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20">
+        <v>38</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21">
       <c r="A5" s="4" t="s">
         <v>42</v>
       </c>
@@ -13507,8 +13524,11 @@
       <c r="T5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:20">
+      <c r="U5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21">
       <c r="A6" s="4" t="s">
         <v>43</v>
       </c>
@@ -13550,11 +13570,12 @@
       <c r="Q6" s="5"/>
       <c r="R6" s="5"/>
       <c r="S6" s="5"/>
-      <c r="T6" s="5" t="s">
+      <c r="T6" s="5"/>
+      <c r="U6" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="42" customHeight="1">
+    <row r="7" spans="1:21" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>52</v>
       </c>
@@ -13577,9 +13598,10 @@
       <c r="R7" s="6"/>
       <c r="S7" s="6"/>
       <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
@@ -13592,6 +13614,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, ExactOfficialText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="DuEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactStructured,ExactPublicText,ExactOfficialText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: WeightedCurio, GrandMiracle" promptTitle="DuHexContentKind enum" prompt="Select a value from the dropdown." sqref="P8:P1007">
+      <formula1>"WeightedCurio,GrandMiracle"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13624,7 +13649,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -13648,7 +13673,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -13698,13 +13723,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>132</v>
@@ -13760,13 +13785,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>132</v>
@@ -13822,7 +13847,7 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>38</v>
@@ -14015,7 +14040,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -14039,7 +14064,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -14089,7 +14114,7 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>178</v>
@@ -14098,7 +14123,7 @@
         <v>232</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>146</v>
@@ -14154,7 +14179,7 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>178</v>
@@ -14163,7 +14188,7 @@
         <v>232</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>146</v>
@@ -14219,7 +14244,7 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>38</v>
@@ -14794,7 +14819,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -14818,7 +14843,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -14871,10 +14896,10 @@
         <v>150</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>28</v>
@@ -14930,10 +14955,10 @@
         <v>150</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>28</v>
@@ -15171,7 +15196,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -15195,7 +15220,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -15245,16 +15270,16 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>136</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>119</v>
@@ -15310,16 +15335,16 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>136</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>119</v>
@@ -15375,10 +15400,10 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>38</v>
@@ -15576,7 +15601,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -15600,7 +15625,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -15650,19 +15675,19 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>136</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="U2" s="3" t="s">
         <v>28</v>
@@ -15715,19 +15740,19 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>136</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="U3" s="5" t="s">
         <v>28</v>
@@ -15780,10 +15805,10 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>38</v>
@@ -15981,7 +16006,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -16005,7 +16030,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -16055,7 +16080,7 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>168</v>
@@ -16064,7 +16089,7 @@
         <v>132</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>171</v>
@@ -16120,7 +16145,7 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>168</v>
@@ -16129,7 +16154,7 @@
         <v>132</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>171</v>
@@ -16185,10 +16210,10 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>38</v>
@@ -16386,7 +16411,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -16410,7 +16435,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -16460,13 +16485,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>232</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>28</v>
@@ -16519,13 +16544,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>232</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>28</v>
@@ -16763,7 +16788,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -16787,7 +16812,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -16837,13 +16862,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>28</v>
@@ -16896,13 +16921,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>28</v>
@@ -16955,10 +16980,10 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>38</v>
@@ -17142,7 +17167,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -17166,7 +17191,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -17216,16 +17241,16 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>28</v>
@@ -17278,16 +17303,16 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>28</v>
@@ -17531,7 +17556,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -17555,7 +17580,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -17605,13 +17630,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>28</v>
@@ -17664,13 +17689,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>28</v>
@@ -17906,7 +17931,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -17930,7 +17955,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -17980,13 +18005,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>66</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>28</v>
@@ -18039,13 +18064,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>66</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>28</v>
@@ -18281,7 +18306,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -18305,7 +18330,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -18355,13 +18380,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>66</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>28</v>
@@ -18414,13 +18439,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>66</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>28</v>
@@ -19051,7 +19076,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -19075,7 +19100,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -19125,16 +19150,16 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>28</v>
@@ -19187,16 +19212,16 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>28</v>
@@ -19444,7 +19469,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -19468,7 +19493,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -19518,16 +19543,16 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>171</v>
@@ -19583,16 +19608,16 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>171</v>
@@ -19648,7 +19673,7 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>38</v>
@@ -19847,7 +19872,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -19871,7 +19896,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -19921,7 +19946,7 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>168</v>
@@ -19930,7 +19955,7 @@
         <v>229</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>171</v>
@@ -19986,7 +20011,7 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>168</v>
@@ -19995,7 +20020,7 @@
         <v>229</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>171</v>
@@ -20252,7 +20277,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -20276,7 +20301,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -20326,19 +20351,19 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>119</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="U2" s="3" t="s">
         <v>28</v>
@@ -20391,19 +20416,19 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>119</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="U3" s="5" t="s">
         <v>28</v>
@@ -20456,10 +20481,10 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>38</v>
@@ -20662,7 +20687,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -20686,7 +20711,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -20736,13 +20761,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>28</v>
@@ -20795,13 +20820,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>28</v>
@@ -20854,7 +20879,7 @@
         <v>38</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>38</v>
@@ -21037,7 +21062,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -21061,7 +21086,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -21111,13 +21136,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>28</v>
@@ -21170,13 +21195,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>28</v>
@@ -21412,7 +21437,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -21436,7 +21461,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -21486,13 +21511,13 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>119</v>
@@ -21548,13 +21573,13 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>119</v>
@@ -21801,7 +21826,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -21825,7 +21850,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -21878,10 +21903,10 @@
         <v>93</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>28</v>
@@ -21937,10 +21962,10 @@
         <v>93</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>28</v>
@@ -22177,7 +22202,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -22201,7 +22226,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -22251,7 +22276,7 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>184</v>
@@ -22307,7 +22332,7 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>184</v>

</xml_diff>